<commit_message>
v17-v21: SMB restructure with NAPS Data/Plan tables, Outreach KPI strip, Out Reach Status, HJ Employer ID, Certification Pipeline on-Going with Project + Slab filter, Sub Cluster cards on Home, Community Colleges Source filter, SAHI first-load fix, FY filter on projects, Manpower project narrowing
</commit_message>
<xml_diff>
--- a/data/NAPS Eligible.xlsx
+++ b/data/NAPS Eligible.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Praveen S N\PycharmProjects\website\mis_dashboard\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Praveen SN\PycharmProjects\website\mis_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{993138BE-A589-467A-8A52-CBFB37AA85EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{845643F8-8B89-4010-9992-2D2E1E8C4B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{F9C43D83-64FC-40CD-87CE-7E0985E9721D}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{F9C43D83-64FC-40CD-87CE-7E0985E9721D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -886,19 +886,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{586E6743-F174-4E98-A2EB-3B89BB5B3234}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="59.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="59.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.06640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.06640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -924,7 +924,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -950,7 +950,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -976,7 +976,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1054,7 +1054,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1080,7 +1080,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>51</v>
       </c>
@@ -1184,7 +1184,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>5</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1340,7 +1340,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -1366,7 +1366,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>50</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>24</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -1548,7 +1548,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>35</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -1600,7 +1600,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -1626,7 +1626,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -1678,7 +1678,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>52</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>13</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -1808,7 +1808,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>9</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>47</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>17</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>7</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>16</v>
       </c>
@@ -1988,7 +1988,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>23</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>33</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>12</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>15</v>
       </c>
@@ -2020,7 +2020,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>40</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>41</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>42</v>
       </c>
@@ -2044,7 +2044,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>44</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>46</v>
       </c>
@@ -2060,7 +2060,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>49</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>53</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>55</v>
       </c>

</xml_diff>

<commit_message>
Monthly Demand drill-downs: sourcing popups, QP Match, centre team, cascading filters
</commit_message>
<xml_diff>
--- a/data/NAPS Eligible.xlsx
+++ b/data/NAPS Eligible.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Praveen SN\PycharmProjects\website\mis_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27604F8-8D96-4400-80CA-BD17A9351FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4BCA7E-76C7-4F4F-AA63-F9F2A680F258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{F9C43D83-64FC-40CD-87CE-7E0985E9721D}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$I$66</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="167">
   <si>
     <t>Electric Vehicle Service Technician</t>
   </si>
@@ -281,9 +281,6 @@
     <t>QP Code</t>
   </si>
   <si>
-    <t>Revised QP Code</t>
-  </si>
-  <si>
     <t>NAPS Aligned</t>
   </si>
   <si>
@@ -302,9 +299,6 @@
     <t>SCGJ</t>
   </si>
   <si>
-    <t>SGJ/Q0101</t>
-  </si>
-  <si>
     <t>ELE/Q5901</t>
   </si>
   <si>
@@ -320,9 +314,6 @@
     <t>ASDC</t>
   </si>
   <si>
-    <t>ASC/Q1424</t>
-  </si>
-  <si>
     <t>ASC/Q1429</t>
   </si>
   <si>
@@ -341,33 +332,21 @@
     <t>SSC/Q2210</t>
   </si>
   <si>
-    <t>SSC/Q9006</t>
-  </si>
-  <si>
     <t>SSC/Q2702</t>
   </si>
   <si>
-    <t>ASC/Q1001</t>
-  </si>
-  <si>
     <t>ASC/Q1005</t>
   </si>
   <si>
     <t>8,000-9,000</t>
   </si>
   <si>
-    <t>ASC/Q3501</t>
-  </si>
-  <si>
     <t>ASC/Q3604</t>
   </si>
   <si>
     <t>RASCI</t>
   </si>
   <si>
-    <t>RAS/Q0103</t>
-  </si>
-  <si>
     <t>RAS/Q0104</t>
   </si>
   <si>
@@ -377,15 +356,9 @@
     <t>ESSCI</t>
   </si>
   <si>
-    <t>ELE/Q3301</t>
-  </si>
-  <si>
     <t>CSC/Q0305</t>
   </si>
   <si>
-    <t>ASC/Q1412</t>
-  </si>
-  <si>
     <t>ASC/Q1402</t>
   </si>
   <si>
@@ -422,27 +395,12 @@
     <t>ASC/Q1405</t>
   </si>
   <si>
-    <t>ASC/Q3302</t>
-  </si>
-  <si>
-    <t>ASC/Q3304</t>
-  </si>
-  <si>
-    <t>ASC/Q4401</t>
-  </si>
-  <si>
-    <t>ASC/Q3506</t>
-  </si>
-  <si>
     <t>ASC/Q3101</t>
   </si>
   <si>
     <t>LSSC</t>
   </si>
   <si>
-    <t>LSS /Q5501</t>
-  </si>
-  <si>
     <t>B&amp;WSSC</t>
   </si>
   <si>
@@ -468,9 +426,6 @@
   </si>
   <si>
     <t>CSC/Q0303</t>
-  </si>
-  <si>
-    <t>SSC/Q0909</t>
   </si>
   <si>
     <t xml:space="preserve">SSC Q0929
@@ -489,9 +444,6 @@
     <t>CSC/Q1003 - Greenhouse operator not aligend</t>
   </si>
   <si>
-    <t>CON/Q721</t>
-  </si>
-  <si>
     <t>THSC</t>
   </si>
   <si>
@@ -510,54 +462,27 @@
     <t>AGR/Q4101</t>
   </si>
   <si>
-    <t>AGR/Q4103</t>
-  </si>
-  <si>
     <t>PCSC / CSDCI</t>
   </si>
   <si>
-    <t>PCS/Q5101</t>
-  </si>
-  <si>
     <t>CON/Q0503</t>
   </si>
   <si>
     <t>ASC/Q1411</t>
   </si>
   <si>
-    <t>BWS/Q0201</t>
-  </si>
-  <si>
     <t>BWS/Q0202</t>
   </si>
   <si>
-    <t>BWS/Q0401</t>
-  </si>
-  <si>
-    <t>SSC/Q9103</t>
-  </si>
-  <si>
-    <t>MES/Q0705</t>
-  </si>
-  <si>
     <t>Life Skills / Entrep.</t>
   </si>
   <si>
     <t>LSC</t>
   </si>
   <si>
-    <t>LSC/Q2101</t>
-  </si>
-  <si>
     <t>LSC/Q0101</t>
   </si>
   <si>
-    <t>CSC/Q0103</t>
-  </si>
-  <si>
-    <t>CSC/Q0204</t>
-  </si>
-  <si>
     <t>PSC</t>
   </si>
   <si>
@@ -576,21 +501,9 @@
     <t>MEPSC</t>
   </si>
   <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>AMH/Q1948</t>
-  </si>
-  <si>
-    <t>AMH/Q 1001</t>
-  </si>
-  <si>
     <t>ASC/Q6411-Automotive Additive Manufacturing Technician</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
     <t>RAS/Q0102</t>
   </si>
   <si>
@@ -600,31 +513,37 @@
     <t>PSSC</t>
   </si>
   <si>
-    <t>PSS/Q3101</t>
-  </si>
-  <si>
-    <t>PSS/Q6001</t>
-  </si>
-  <si>
     <t>Handicrafts</t>
   </si>
   <si>
     <t>GJSCI</t>
   </si>
   <si>
-    <t xml:space="preserve"> G&amp;J/Q2301</t>
-  </si>
-  <si>
-    <t>SSC/Q0501</t>
-  </si>
-  <si>
-    <t>SSC/Q0503</t>
-  </si>
-  <si>
     <t>HCSSC</t>
   </si>
   <si>
-    <t>HCS/Q8705</t>
+    <t xml:space="preserve">ASC/Q3302 </t>
+  </si>
+  <si>
+    <t>BWS/Q0403</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSS/Q6001 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SSC/Q0503 </t>
+  </si>
+  <si>
+    <t>MES/Q0706</t>
+  </si>
+  <si>
+    <t>ELE/Q0102</t>
+  </si>
+  <si>
+    <t>TSC/Q0114</t>
+  </si>
+  <si>
+    <t>AMH/Q1001</t>
   </si>
 </sst>
 </file>
@@ -660,7 +579,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -670,6 +589,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -715,7 +640,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -726,6 +651,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1071,14 +997,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{586E6743-F174-4E98-A2EB-3B89BB5B3234}">
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:I66"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="7" max="7" width="10.86328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.53125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.46484375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>75</v>
       </c>
@@ -1106,11 +1038,8 @@
       <c r="I1" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>30</v>
       </c>
@@ -1118,31 +1047,28 @@
         <v>52</v>
       </c>
       <c r="C2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" t="s">
         <v>84</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>85</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" t="s">
         <v>86</v>
       </c>
-      <c r="F2" t="s">
-        <v>87</v>
-      </c>
-      <c r="G2" t="s">
-        <v>52</v>
-      </c>
-      <c r="H2" t="s">
-        <v>54</v>
-      </c>
       <c r="I2" t="s">
-        <v>88</v>
-      </c>
-      <c r="J2" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -1150,31 +1076,28 @@
         <v>52</v>
       </c>
       <c r="C3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E3" t="s">
         <v>90</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" t="s">
         <v>91</v>
       </c>
-      <c r="E3" t="s">
+      <c r="I3" t="s">
         <v>92</v>
       </c>
-      <c r="F3" t="s">
-        <v>93</v>
-      </c>
-      <c r="G3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H3" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" t="s">
-        <v>94</v>
-      </c>
-      <c r="J3" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -1185,25 +1108,25 @@
         <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
-      </c>
-      <c r="G4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I4" t="s">
-        <v>94</v>
-      </c>
-      <c r="J4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1214,25 +1137,25 @@
         <v>53</v>
       </c>
       <c r="D5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
-      </c>
-      <c r="G5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I5" t="s">
-        <v>94</v>
-      </c>
-      <c r="J5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>31</v>
       </c>
@@ -1243,28 +1166,25 @@
         <v>53</v>
       </c>
       <c r="D6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" t="s">
         <v>96</v>
       </c>
-      <c r="E6" t="s">
-        <v>99</v>
-      </c>
-      <c r="F6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="F6" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H6" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I6" t="s">
-        <v>94</v>
-      </c>
-      <c r="J6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>32</v>
       </c>
@@ -1272,31 +1192,28 @@
         <v>52</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E7" t="s">
-        <v>101</v>
-      </c>
-      <c r="F7" t="s">
-        <v>102</v>
-      </c>
-      <c r="G7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H7" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I7" t="s">
-        <v>88</v>
-      </c>
-      <c r="J7" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>33</v>
       </c>
@@ -1304,31 +1221,28 @@
         <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D8" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E8" t="s">
-        <v>104</v>
-      </c>
-      <c r="F8" t="s">
-        <v>105</v>
-      </c>
-      <c r="G8" t="s">
+        <v>99</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I8" t="s">
-        <v>88</v>
-      </c>
-      <c r="J8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -1339,28 +1253,25 @@
         <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E9" t="s">
-        <v>107</v>
-      </c>
-      <c r="F9" t="s">
-        <v>108</v>
-      </c>
-      <c r="G9" t="s">
+        <v>101</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I9" t="s">
-        <v>88</v>
-      </c>
-      <c r="J9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>34</v>
       </c>
@@ -1368,31 +1279,28 @@
         <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D10" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="E10" t="s">
-        <v>111</v>
-      </c>
-      <c r="F10" t="s">
-        <v>112</v>
-      </c>
-      <c r="G10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H10" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I10" t="s">
-        <v>88</v>
-      </c>
-      <c r="J10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>35</v>
       </c>
@@ -1400,31 +1308,28 @@
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D11" t="s">
+        <v>89</v>
+      </c>
+      <c r="E11" t="s">
+        <v>105</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" t="s">
         <v>91</v>
       </c>
-      <c r="E11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" t="s">
-        <v>114</v>
-      </c>
-      <c r="G11" t="s">
-        <v>52</v>
-      </c>
-      <c r="H11" t="s">
-        <v>52</v>
-      </c>
       <c r="I11" t="s">
-        <v>94</v>
-      </c>
-      <c r="J11" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>36</v>
       </c>
@@ -1432,31 +1337,28 @@
         <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E12" t="s">
-        <v>104</v>
-      </c>
-      <c r="F12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G12" t="s">
+        <v>99</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H12" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I12" t="s">
-        <v>88</v>
-      </c>
-      <c r="J12" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
@@ -1467,28 +1369,25 @@
         <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E13" t="s">
-        <v>115</v>
-      </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
-      <c r="G13" t="s">
+        <v>106</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H13" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I13" t="s">
-        <v>94</v>
-      </c>
-      <c r="J13" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
@@ -1499,28 +1398,25 @@
         <v>53</v>
       </c>
       <c r="D14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E14" t="s">
-        <v>116</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H14" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I14" t="s">
-        <v>94</v>
-      </c>
-      <c r="J14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>18</v>
       </c>
@@ -1528,31 +1424,28 @@
         <v>52</v>
       </c>
       <c r="C15" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="E15" t="s">
-        <v>119</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15" t="s">
-        <v>52</v>
+        <v>110</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H15" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I15" t="s">
-        <v>120</v>
-      </c>
-      <c r="J15" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
         <v>62</v>
       </c>
@@ -1560,31 +1453,28 @@
         <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D16" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E16" t="s">
-        <v>123</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16" t="s">
-        <v>52</v>
+        <v>114</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H16" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="I16" t="s">
-        <v>124</v>
-      </c>
-      <c r="J16" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>63</v>
       </c>
@@ -1592,31 +1482,28 @@
         <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E17" t="s">
-        <v>125</v>
-      </c>
-      <c r="F17" t="s">
-        <v>126</v>
-      </c>
-      <c r="G17" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H17" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I17" t="s">
-        <v>88</v>
-      </c>
-      <c r="J17" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>64</v>
       </c>
@@ -1624,31 +1511,28 @@
         <v>52</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D18" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E18" t="s">
-        <v>127</v>
-      </c>
-      <c r="F18" t="s">
-        <v>128</v>
-      </c>
-      <c r="G18" t="s">
+        <v>159</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H18" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I18" t="s">
-        <v>88</v>
-      </c>
-      <c r="J18" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A19" s="3" t="s">
         <v>65</v>
       </c>
@@ -1656,31 +1540,28 @@
         <v>52</v>
       </c>
       <c r="C19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E19" t="s">
-        <v>129</v>
-      </c>
-      <c r="F19" t="s">
-        <v>130</v>
-      </c>
-      <c r="G19" t="s">
+        <v>117</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H19" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I19" t="s">
-        <v>88</v>
-      </c>
-      <c r="J19" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>66</v>
       </c>
@@ -1688,31 +1569,28 @@
         <v>52</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D20" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>123</v>
-      </c>
-      <c r="F20" t="s">
-        <v>132</v>
-      </c>
-      <c r="G20" t="s">
-        <v>52</v>
+        <v>114</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H20" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="I20" t="s">
-        <v>124</v>
-      </c>
-      <c r="J20" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>6</v>
       </c>
@@ -1723,28 +1601,25 @@
         <v>55</v>
       </c>
       <c r="D21" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E21" t="s">
-        <v>134</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
-      <c r="G21" t="s">
-        <v>52</v>
+        <v>120</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H21" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I21" t="s">
-        <v>120</v>
-      </c>
-      <c r="J21" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
         <v>67</v>
       </c>
@@ -1752,28 +1627,28 @@
         <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="D22" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="E22" t="s">
-        <v>137</v>
-      </c>
-      <c r="G22" t="s">
+        <v>123</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H22" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I22" t="s">
-        <v>88</v>
-      </c>
-      <c r="J22" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
         <v>68</v>
       </c>
@@ -1781,28 +1656,28 @@
         <v>52</v>
       </c>
       <c r="C23" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>138</v>
-      </c>
-      <c r="G23" t="s">
+        <v>124</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H23" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I23" t="s">
-        <v>94</v>
-      </c>
-      <c r="J23" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>46</v>
       </c>
@@ -1810,28 +1685,28 @@
         <v>52</v>
       </c>
       <c r="C24" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D24" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E24" t="s">
-        <v>141</v>
-      </c>
-      <c r="G24" t="s">
+        <v>127</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H24" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I24" t="s">
-        <v>88</v>
-      </c>
-      <c r="J24" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
         <v>28</v>
       </c>
@@ -1842,28 +1717,25 @@
         <v>53</v>
       </c>
       <c r="D25" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E25" t="s">
-        <v>142</v>
-      </c>
-      <c r="F25" t="s">
-        <v>143</v>
-      </c>
-      <c r="G25" t="s">
+        <v>128</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H25" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I25" t="s">
-        <v>94</v>
-      </c>
-      <c r="J25" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>9</v>
       </c>
@@ -1871,31 +1743,28 @@
         <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E26" t="s">
-        <v>144</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26" t="s">
-        <v>52</v>
+        <v>129</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H26" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="I26" t="s">
-        <v>124</v>
-      </c>
-      <c r="J26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A27" s="3" t="s">
         <v>1</v>
       </c>
@@ -1906,25 +1775,25 @@
         <v>53</v>
       </c>
       <c r="D27" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>145</v>
-      </c>
-      <c r="G27" t="s">
+        <v>130</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H27" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I27" t="s">
-        <v>94</v>
-      </c>
-      <c r="J27" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A28" s="3" t="s">
         <v>37</v>
       </c>
@@ -1932,31 +1801,28 @@
         <v>52</v>
       </c>
       <c r="C28" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D28" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="E28" t="s">
-        <v>147</v>
-      </c>
-      <c r="F28" t="s">
-        <v>148</v>
-      </c>
-      <c r="G28" t="s">
+        <v>132</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G28" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H28" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I28" t="s">
-        <v>88</v>
-      </c>
-      <c r="J28" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1967,25 +1833,25 @@
         <v>60</v>
       </c>
       <c r="D29" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="E29" t="s">
-        <v>150</v>
-      </c>
-      <c r="G29" t="s">
+        <v>134</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H29" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I29" t="s">
-        <v>88</v>
-      </c>
-      <c r="J29" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A30" s="3" t="s">
         <v>48</v>
       </c>
@@ -1996,25 +1862,25 @@
         <v>60</v>
       </c>
       <c r="D30" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="E30" t="s">
-        <v>151</v>
-      </c>
-      <c r="G30" t="s">
+        <v>135</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G30" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H30" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I30" t="s">
-        <v>88</v>
-      </c>
-      <c r="J30" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A31" s="3" t="s">
         <v>40</v>
       </c>
@@ -2022,28 +1888,28 @@
         <v>52</v>
       </c>
       <c r="C31" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E31" t="s">
-        <v>141</v>
-      </c>
-      <c r="G31" t="s">
+        <v>127</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H31" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I31" t="s">
-        <v>88</v>
-      </c>
-      <c r="J31" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A32" s="3" t="s">
         <v>2</v>
       </c>
@@ -2051,31 +1917,28 @@
         <v>52</v>
       </c>
       <c r="C32" t="s">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="D32" t="s">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="E32" t="s">
-        <v>154</v>
-      </c>
-      <c r="F32" t="s">
-        <v>155</v>
-      </c>
-      <c r="G32" t="s">
-        <v>52</v>
+        <v>138</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H32" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="I32" t="s">
-        <v>124</v>
-      </c>
-      <c r="J32" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A33" s="3" t="s">
         <v>5</v>
       </c>
@@ -2086,28 +1949,25 @@
         <v>58</v>
       </c>
       <c r="D33" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="E33" t="s">
-        <v>157</v>
-      </c>
-      <c r="F33" t="s">
-        <v>158</v>
-      </c>
-      <c r="G33" t="s">
-        <v>52</v>
+        <v>140</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H33" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I33" t="s">
-        <v>120</v>
-      </c>
-      <c r="J33" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
         <v>7</v>
       </c>
@@ -2115,31 +1975,28 @@
         <v>52</v>
       </c>
       <c r="C34" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D34" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" t="s">
+        <v>141</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H34" t="s">
         <v>91</v>
       </c>
-      <c r="E34" t="s">
-        <v>159</v>
-      </c>
-      <c r="F34">
-        <v>0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>52</v>
-      </c>
-      <c r="H34" t="s">
-        <v>52</v>
-      </c>
       <c r="I34" t="s">
-        <v>94</v>
-      </c>
-      <c r="J34" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
         <v>10</v>
       </c>
@@ -2150,28 +2007,25 @@
         <v>55</v>
       </c>
       <c r="D35" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E35" t="s">
-        <v>160</v>
-      </c>
-      <c r="F35" t="s">
-        <v>161</v>
-      </c>
-      <c r="G35" t="s">
-        <v>52</v>
+        <v>142</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H35" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I35" t="s">
-        <v>120</v>
-      </c>
-      <c r="J35" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -2182,28 +2036,25 @@
         <v>55</v>
       </c>
       <c r="D36" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E36" t="s">
-        <v>162</v>
-      </c>
-      <c r="F36">
-        <v>0</v>
-      </c>
-      <c r="G36" t="s">
-        <v>52</v>
+        <v>160</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H36" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I36" t="s">
-        <v>120</v>
-      </c>
-      <c r="J36" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A37" s="3" t="s">
         <v>13</v>
       </c>
@@ -2214,28 +2065,25 @@
         <v>53</v>
       </c>
       <c r="D37" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E37" t="s">
         <v>163</v>
       </c>
-      <c r="F37" t="s">
-        <v>164</v>
-      </c>
-      <c r="G37" t="s">
+      <c r="F37" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G37" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H37" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I37" t="s">
-        <v>94</v>
-      </c>
-      <c r="J37" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A38" s="3" t="s">
         <v>14</v>
       </c>
@@ -2243,31 +2091,28 @@
         <v>54</v>
       </c>
       <c r="C38" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="D38" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E38" t="s">
-        <v>89</v>
-      </c>
-      <c r="F38">
-        <v>0</v>
-      </c>
-      <c r="G38" t="s">
+        <v>87</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G38" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H38" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I38" t="s">
-        <v>89</v>
-      </c>
-      <c r="J38" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
         <v>15</v>
       </c>
@@ -2278,28 +2123,25 @@
         <v>56</v>
       </c>
       <c r="D39" t="s">
-        <v>166</v>
+        <v>144</v>
       </c>
       <c r="E39" t="s">
-        <v>167</v>
-      </c>
-      <c r="F39" t="s">
-        <v>168</v>
-      </c>
-      <c r="G39" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G39" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H39" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I39" t="s">
-        <v>88</v>
-      </c>
-      <c r="J39" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A40" s="3" t="s">
         <v>16</v>
       </c>
@@ -2307,31 +2149,28 @@
         <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D40" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="E40" t="s">
-        <v>169</v>
-      </c>
-      <c r="F40" t="s">
-        <v>170</v>
-      </c>
-      <c r="G40" t="s">
+        <v>164</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G40" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H40" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I40" t="s">
-        <v>88</v>
-      </c>
-      <c r="J40" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A41" s="3" t="s">
         <v>17</v>
       </c>
@@ -2342,25 +2181,25 @@
         <v>58</v>
       </c>
       <c r="D41" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="E41" t="s">
-        <v>172</v>
-      </c>
-      <c r="G41" t="s">
-        <v>52</v>
+        <v>147</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H41" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I41" t="s">
-        <v>120</v>
-      </c>
-      <c r="J41" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
         <v>19</v>
       </c>
@@ -2371,25 +2210,25 @@
         <v>55</v>
       </c>
       <c r="D42" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E42" t="s">
-        <v>173</v>
-      </c>
-      <c r="G42" t="s">
-        <v>52</v>
+        <v>148</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H42" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I42" t="s">
-        <v>120</v>
-      </c>
-      <c r="J42" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A43" s="3" t="s">
         <v>20</v>
       </c>
@@ -2400,25 +2239,25 @@
         <v>59</v>
       </c>
       <c r="D43" t="s">
-        <v>174</v>
+        <v>149</v>
       </c>
       <c r="E43" t="s">
-        <v>175</v>
-      </c>
-      <c r="G43" t="s">
-        <v>52</v>
+        <v>150</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H43" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="I43" t="s">
-        <v>88</v>
-      </c>
-      <c r="J43" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A44" s="3" t="s">
         <v>21</v>
       </c>
@@ -2426,31 +2265,28 @@
         <v>54</v>
       </c>
       <c r="C44" t="s">
+        <v>143</v>
+      </c>
+      <c r="D44" t="s">
+        <v>151</v>
+      </c>
+      <c r="E44" t="s">
         <v>165</v>
       </c>
-      <c r="D44" t="s">
-        <v>176</v>
-      </c>
-      <c r="E44" t="s">
-        <v>177</v>
-      </c>
-      <c r="F44">
-        <v>0</v>
-      </c>
-      <c r="G44" t="s">
+      <c r="F44" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G44" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H44" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I44" t="s">
-        <v>89</v>
-      </c>
-      <c r="J44" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2458,31 +2294,28 @@
         <v>54</v>
       </c>
       <c r="C45" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D45" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E45" t="s">
-        <v>178</v>
-      </c>
-      <c r="F45" t="s">
-        <v>179</v>
-      </c>
-      <c r="G45" t="s">
+        <v>166</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G45" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H45" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I45" t="s">
-        <v>89</v>
-      </c>
-      <c r="J45" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A46" s="3" t="s">
         <v>24</v>
       </c>
@@ -2490,31 +2323,28 @@
         <v>52</v>
       </c>
       <c r="C46" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D46" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E46" t="s">
-        <v>123</v>
-      </c>
-      <c r="F46">
-        <v>0</v>
-      </c>
-      <c r="G46" t="s">
-        <v>52</v>
+        <v>114</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H46" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="I46" t="s">
-        <v>124</v>
-      </c>
-      <c r="J46" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
         <v>25</v>
       </c>
@@ -2522,31 +2352,28 @@
         <v>52</v>
       </c>
       <c r="C47" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E47" t="s">
-        <v>180</v>
-      </c>
-      <c r="F47" t="s">
-        <v>181</v>
-      </c>
-      <c r="G47" t="s">
+        <v>152</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G47" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H47" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I47" t="s">
-        <v>88</v>
-      </c>
-      <c r="J47" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A48" s="3" t="s">
         <v>26</v>
       </c>
@@ -2557,28 +2384,25 @@
         <v>57</v>
       </c>
       <c r="D48" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="E48" t="s">
-        <v>182</v>
-      </c>
-      <c r="F48" t="s">
-        <v>108</v>
-      </c>
-      <c r="G48" t="s">
+        <v>153</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G48" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H48" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I48" t="s">
-        <v>88</v>
-      </c>
-      <c r="J48" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A49" s="3" t="s">
         <v>29</v>
       </c>
@@ -2586,31 +2410,28 @@
         <v>52</v>
       </c>
       <c r="C49" t="s">
-        <v>183</v>
+        <v>154</v>
       </c>
       <c r="D49" t="s">
-        <v>184</v>
+        <v>155</v>
       </c>
       <c r="E49" t="s">
-        <v>185</v>
-      </c>
-      <c r="F49" t="s">
-        <v>186</v>
-      </c>
-      <c r="G49" t="s">
+        <v>161</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G49" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H49" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I49" t="s">
-        <v>88</v>
-      </c>
-      <c r="J49" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A50" s="3" t="s">
         <v>38</v>
       </c>
@@ -2618,31 +2439,28 @@
         <v>54</v>
       </c>
       <c r="C50" t="s">
-        <v>187</v>
+        <v>156</v>
       </c>
       <c r="D50" t="s">
-        <v>188</v>
+        <v>157</v>
       </c>
       <c r="E50" t="s">
-        <v>177</v>
-      </c>
-      <c r="F50" t="s">
-        <v>189</v>
-      </c>
-      <c r="G50" t="s">
+        <v>165</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G50" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H50" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I50" t="s">
-        <v>89</v>
-      </c>
-      <c r="J50" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
         <v>39</v>
       </c>
@@ -2653,28 +2471,25 @@
         <v>53</v>
       </c>
       <c r="D51" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E51" t="s">
-        <v>190</v>
-      </c>
-      <c r="F51" t="s">
-        <v>191</v>
-      </c>
-      <c r="G51" t="s">
+        <v>162</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G51" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H51" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I51" t="s">
-        <v>94</v>
-      </c>
-      <c r="J51" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A52" s="3" t="s">
         <v>41</v>
       </c>
@@ -2682,31 +2497,28 @@
         <v>54</v>
       </c>
       <c r="C52" t="s">
-        <v>187</v>
+        <v>156</v>
       </c>
       <c r="D52" t="s">
-        <v>192</v>
+        <v>158</v>
       </c>
       <c r="E52" t="s">
-        <v>177</v>
-      </c>
-      <c r="F52" t="s">
-        <v>193</v>
-      </c>
-      <c r="G52" t="s">
+        <v>165</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G52" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H52" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I52" t="s">
-        <v>89</v>
-      </c>
-      <c r="J52" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A53" s="3" t="s">
         <v>42</v>
       </c>
@@ -2714,28 +2526,28 @@
         <v>54</v>
       </c>
       <c r="C53" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D53" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="E53" t="s">
-        <v>177</v>
-      </c>
-      <c r="G53" t="s">
+        <v>165</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G53" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H53" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I53" t="s">
-        <v>89</v>
-      </c>
-      <c r="J53" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A54" s="3" t="s">
         <v>43</v>
       </c>
@@ -2743,31 +2555,28 @@
         <v>52</v>
       </c>
       <c r="C54" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D54" t="s">
+        <v>89</v>
+      </c>
+      <c r="E54" t="s">
+        <v>141</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" t="s">
         <v>91</v>
       </c>
-      <c r="E54" t="s">
-        <v>159</v>
-      </c>
-      <c r="F54">
-        <v>0</v>
-      </c>
-      <c r="G54" t="s">
-        <v>52</v>
-      </c>
-      <c r="H54" t="s">
-        <v>52</v>
-      </c>
       <c r="I54" t="s">
-        <v>94</v>
-      </c>
-      <c r="J54" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A55" s="3" t="s">
         <v>44</v>
       </c>
@@ -2778,28 +2587,25 @@
         <v>58</v>
       </c>
       <c r="D55" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="E55" t="s">
-        <v>157</v>
-      </c>
-      <c r="F55" t="s">
-        <v>158</v>
-      </c>
-      <c r="G55" t="s">
-        <v>52</v>
+        <v>140</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H55" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I55" t="s">
-        <v>120</v>
-      </c>
-      <c r="J55" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A56" s="3" t="s">
         <v>45</v>
       </c>
@@ -2807,31 +2613,28 @@
         <v>52</v>
       </c>
       <c r="C56" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D56" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E56" t="s">
-        <v>125</v>
-      </c>
-      <c r="F56" t="s">
-        <v>126</v>
-      </c>
-      <c r="G56" t="s">
+        <v>116</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G56" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H56" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I56" t="s">
-        <v>88</v>
-      </c>
-      <c r="J56" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A57" s="3" t="s">
         <v>47</v>
       </c>
@@ -2839,31 +2642,28 @@
         <v>52</v>
       </c>
       <c r="C57" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D57" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E57" t="s">
-        <v>104</v>
-      </c>
-      <c r="F57" t="s">
-        <v>105</v>
-      </c>
-      <c r="G57" t="s">
+        <v>99</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G57" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H57" t="s">
-        <v>52</v>
+        <v>86</v>
       </c>
       <c r="I57" t="s">
-        <v>88</v>
-      </c>
-      <c r="J57" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A58" s="3" t="s">
         <v>49</v>
       </c>
@@ -2874,28 +2674,25 @@
         <v>53</v>
       </c>
       <c r="D58" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E58" t="s">
-        <v>116</v>
-      </c>
-      <c r="F58" t="s">
-        <v>145</v>
-      </c>
-      <c r="G58" t="s">
+        <v>107</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G58" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H58" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I58" t="s">
-        <v>94</v>
-      </c>
-      <c r="J58" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A59" s="3" t="s">
         <v>50</v>
       </c>
@@ -2903,31 +2700,28 @@
         <v>52</v>
       </c>
       <c r="C59" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="D59" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="E59" t="s">
-        <v>138</v>
-      </c>
-      <c r="F59">
-        <v>0</v>
-      </c>
-      <c r="G59" t="s">
+        <v>124</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G59" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H59" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I59" t="s">
-        <v>94</v>
-      </c>
-      <c r="J59" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
         <v>69</v>
       </c>
@@ -2938,28 +2732,25 @@
         <v>53</v>
       </c>
       <c r="D60" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E60" t="s">
         <v>163</v>
       </c>
-      <c r="F60" t="s">
-        <v>164</v>
-      </c>
-      <c r="G60" t="s">
+      <c r="F60" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G60" s="4" t="s">
         <v>52</v>
       </c>
       <c r="H60" t="s">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="I60" t="s">
-        <v>94</v>
-      </c>
-      <c r="J60" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A61" s="3" t="s">
         <v>51</v>
       </c>
@@ -2967,28 +2758,28 @@
         <v>54</v>
       </c>
       <c r="C61" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="D61" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E61" t="s">
-        <v>89</v>
-      </c>
-      <c r="G61" t="s">
+        <v>87</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G61" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H61" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I61" t="s">
-        <v>89</v>
-      </c>
-      <c r="J61" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A62" s="3" t="s">
         <v>70</v>
       </c>
@@ -2999,25 +2790,25 @@
         <v>55</v>
       </c>
       <c r="D62" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E62" t="s">
-        <v>134</v>
-      </c>
-      <c r="G62" t="s">
-        <v>52</v>
+        <v>120</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="H62" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="I62" t="s">
-        <v>120</v>
-      </c>
-      <c r="J62" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A63" s="3" t="s">
         <v>71</v>
       </c>
@@ -3028,25 +2819,25 @@
         <v>53</v>
       </c>
       <c r="D63" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E63" t="s">
-        <v>89</v>
-      </c>
-      <c r="G63" t="s">
+        <v>87</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G63" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H63" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I63" t="s">
-        <v>89</v>
-      </c>
-      <c r="J63" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
         <v>72</v>
       </c>
@@ -3054,28 +2845,28 @@
         <v>54</v>
       </c>
       <c r="C64" t="s">
+        <v>143</v>
+      </c>
+      <c r="D64" t="s">
+        <v>151</v>
+      </c>
+      <c r="E64" t="s">
         <v>165</v>
       </c>
-      <c r="D64" t="s">
-        <v>176</v>
-      </c>
-      <c r="E64" t="s">
-        <v>177</v>
-      </c>
-      <c r="G64" t="s">
+      <c r="F64" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G64" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H64" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I64" t="s">
-        <v>89</v>
-      </c>
-      <c r="J64" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A65" s="3" t="s">
         <v>73</v>
       </c>
@@ -3083,31 +2874,28 @@
         <v>54</v>
       </c>
       <c r="C65" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="D65" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E65" t="s">
-        <v>89</v>
-      </c>
-      <c r="F65">
-        <v>0</v>
-      </c>
-      <c r="G65" t="s">
+        <v>87</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G65" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H65" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I65" t="s">
-        <v>89</v>
-      </c>
-      <c r="J65" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.45">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A66" s="3" t="s">
         <v>74</v>
       </c>
@@ -3115,28 +2903,25 @@
         <v>54</v>
       </c>
       <c r="C66" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="D66" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E66" t="s">
-        <v>89</v>
-      </c>
-      <c r="F66">
-        <v>0</v>
-      </c>
-      <c r="G66" t="s">
+        <v>87</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G66" s="4" t="s">
         <v>54</v>
       </c>
       <c r="H66" t="s">
-        <v>54</v>
+        <v>87</v>
       </c>
       <c r="I66" t="s">
-        <v>89</v>
-      </c>
-      <c r="J66" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Batch sourcing tables, Projects_FY filter, FY-total actuals, cleanup
</commit_message>
<xml_diff>
--- a/data/NAPS Eligible.xlsx
+++ b/data/NAPS Eligible.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Praveen SN\PycharmProjects\website\mis_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4BCA7E-76C7-4F4F-AA63-F9F2A680F258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{327A7DF0-406A-45F0-BE9A-31653FE0BDC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{F9C43D83-64FC-40CD-87CE-7E0985E9721D}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="170">
   <si>
     <t>Electric Vehicle Service Technician</t>
   </si>
@@ -544,13 +544,22 @@
   </si>
   <si>
     <t>AMH/Q1001</t>
+  </si>
+  <si>
+    <t>Waste to Use</t>
+  </si>
+  <si>
+    <t>Automotive Assembly Operator - 4 Wheelers</t>
+  </si>
+  <si>
+    <t>CNC Operator</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -572,6 +581,14 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -640,7 +657,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -652,6 +669,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -997,9 +1017,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{586E6743-F174-4E98-A2EB-3B89BB5B3234}">
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
+    <col min="1" max="1" width="46.796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.3984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.53125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
@@ -2924,6 +2945,93 @@
         <v>87</v>
       </c>
     </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A67" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="B67" t="s">
+        <v>54</v>
+      </c>
+      <c r="C67" t="s">
+        <v>143</v>
+      </c>
+      <c r="D67" t="s">
+        <v>87</v>
+      </c>
+      <c r="E67" t="s">
+        <v>87</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H67" t="s">
+        <v>87</v>
+      </c>
+      <c r="I67" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A68" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B68" t="s">
+        <v>52</v>
+      </c>
+      <c r="C68" t="s">
+        <v>88</v>
+      </c>
+      <c r="D68" t="s">
+        <v>89</v>
+      </c>
+      <c r="E68" t="s">
+        <v>99</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H68" t="s">
+        <v>86</v>
+      </c>
+      <c r="I68" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A69" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="B69" t="s">
+        <v>52</v>
+      </c>
+      <c r="C69" t="s">
+        <v>88</v>
+      </c>
+      <c r="D69" t="s">
+        <v>89</v>
+      </c>
+      <c r="E69" t="s">
+        <v>99</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H69" t="s">
+        <v>86</v>
+      </c>
+      <c r="I69" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="A1:B1">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>